<commit_message>
Macierz CX: usuniete kolumny Status prognozy i Initiative ID (arkusz i konwerter)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/macierz_CX.xlsx
+++ b/macierz_CX.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Dane" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Macierz CX'!$A$1:$AB$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Macierz CX'!$A$1:$Z$61</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -722,7 +722,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB61"/>
+  <dimension ref="A1:Z61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="36.75" customHeight="1"/>
   <cols>
     <col width="8.7109375" customWidth="1" style="33" min="1" max="1"/>
@@ -747,10 +747,8 @@
     <col width="14" customWidth="1" style="34" min="22" max="22"/>
     <col width="14" customWidth="1" style="34" min="23" max="23"/>
     <col width="14" customWidth="1" style="34" min="24" max="24"/>
-    <col width="14" customWidth="1" style="34" min="25" max="16384"/>
-    <col width="13" customWidth="1" min="26" max="26"/>
-    <col width="25.43" customWidth="1" min="27" max="27"/>
-    <col width="66.86" customWidth="1" min="28" max="28"/>
+    <col width="25.43" customWidth="1" style="34" min="25" max="16384"/>
+    <col width="66.86" customWidth="1" min="26" max="26"/>
   </cols>
   <sheetData>
     <row r="1" ht="36.75" customFormat="1" customHeight="1" s="38">
@@ -876,20 +874,10 @@
       </c>
       <c r="Y1" s="38" t="inlineStr">
         <is>
-          <t>Status prognozy</t>
+          <t>Uzasadnienie z danych</t>
         </is>
       </c>
       <c r="Z1" s="38" t="inlineStr">
-        <is>
-          <t>Initiative ID</t>
-        </is>
-      </c>
-      <c r="AA1" s="38" t="inlineStr">
-        <is>
-          <t>Uzasadnienie z danych</t>
-        </is>
-      </c>
-      <c r="AB1" s="38" t="inlineStr">
         <is>
           <t>Źródło insightu</t>
         </is>
@@ -993,12 +981,6 @@
       <c r="X2" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="Y2" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z2" s="37" t="n"/>
     </row>
     <row r="3" ht="36.75" customHeight="1">
       <c r="A3" s="17" t="inlineStr">
@@ -1098,12 +1080,6 @@
       <c r="X3" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="Y3" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z3" s="37" t="n"/>
     </row>
     <row r="4" ht="36.75" customHeight="1">
       <c r="A4" s="17" t="inlineStr">
@@ -1203,12 +1179,6 @@
       <c r="X4" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="Y4" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z4" s="37" t="n"/>
     </row>
     <row r="5" ht="36.75" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
@@ -1308,12 +1278,6 @@
       <c r="X5" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="Y5" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z5" s="37" t="n"/>
     </row>
     <row r="6" ht="36.75" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
@@ -1413,13 +1377,7 @@
       <c r="X6" s="37" t="n">
         <v>3</v>
       </c>
-      <c r="Y6" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z6" s="37" t="n"/>
-      <c r="AA6" s="34" t="inlineStr">
+      <c r="Y6" s="34" t="inlineStr">
         <is>
           <t>Leady z formularza jazdy testowej są obsługiwane przez CRC w SLA poniżej 8 minut od poniedziałku do piątku; monitorowany jest kontakt i skuteczność źródła.</t>
         </is>
@@ -1523,12 +1481,6 @@
       <c r="X7" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="Y7" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z7" s="37" t="n"/>
     </row>
     <row r="8" ht="36.75" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
@@ -1618,12 +1570,6 @@
       <c r="X8" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="Y8" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z8" s="37" t="n"/>
     </row>
     <row r="9" ht="36.75" customHeight="1">
       <c r="A9" s="19" t="inlineStr">
@@ -1723,13 +1669,7 @@
       <c r="X9" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="Y9" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z9" s="37" t="n"/>
-      <c r="AA9" s="34" t="inlineStr">
+      <c r="Y9" s="34" t="inlineStr">
         <is>
           <t>CRC kontaktuje klienta, umawia jazdę testową i przekazuje dealerowi zweryfikowany lead; monitoring pokazuje kontakt oraz jakość źródła.</t>
         </is>
@@ -1823,13 +1763,7 @@
       <c r="X10" s="37" t="n">
         <v>3</v>
       </c>
-      <c r="Y10" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z10" s="37" t="n"/>
-      <c r="AA10" s="34" t="inlineStr">
+      <c r="Y10" s="34" t="inlineStr">
         <is>
           <t>Klient wykonał pierwszy aktywny krok i oczekuje odpowiedzi. Problem pojawia się przy braku reakcji.</t>
         </is>
@@ -1933,12 +1867,6 @@
       <c r="X11" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="Y11" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z11" s="37" t="n"/>
     </row>
     <row r="12" ht="36.75" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
@@ -1961,11 +1889,6 @@
           <t>TP005</t>
         </is>
       </c>
-      <c r="Y12" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
     </row>
     <row r="13" ht="36.75" customHeight="1">
       <c r="A13" s="19" t="inlineStr">
@@ -2065,13 +1988,7 @@
       <c r="X13" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="Y13" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z13" s="37" t="n"/>
-      <c r="AA13" s="34" t="inlineStr">
+      <c r="Y13" s="34" t="inlineStr">
         <is>
           <t>Proces jest centralny i personalizuje kolejność modeli oraz komunikaty według zachowania z poprzednich wizyt; dla jednego komunikatu testowanych jest nawet pięć CTA.</t>
         </is>
@@ -2165,13 +2082,7 @@
       <c r="X14" s="37" t="n">
         <v>0.5</v>
       </c>
-      <c r="Y14" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z14" s="37" t="n"/>
-      <c r="AA14" s="34" t="inlineStr">
+      <c r="Y14" s="34" t="inlineStr">
         <is>
           <t>Emocja zależy od szybkości kontaktu. Dealerzy wskazują problem z oddzwanianiem.</t>
         </is>
@@ -2275,13 +2186,7 @@
       <c r="X15" s="37" t="n">
         <v>5</v>
       </c>
-      <c r="Y15" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z15" s="37" t="n"/>
-      <c r="AA15" s="34" t="inlineStr">
+      <c r="Y15" s="34" t="inlineStr">
         <is>
           <t>Klienci bardzo często pozytywnie oceniają kompetencje i podejście handlowców.</t>
         </is>
@@ -2365,12 +2270,6 @@
       <c r="X16" s="37" t="n">
         <v>5</v>
       </c>
-      <c r="Y16" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z16" s="37" t="n"/>
     </row>
     <row r="17" ht="36.75" customHeight="1">
       <c r="A17" s="19" t="inlineStr">
@@ -2450,12 +2349,6 @@
       <c r="X17" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="Y17" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z17" s="37" t="n"/>
     </row>
     <row r="18" ht="36.75" customHeight="1">
       <c r="A18" s="21" t="inlineStr">
@@ -2555,13 +2448,7 @@
       <c r="X18" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="Y18" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z18" s="37" t="n"/>
-      <c r="AA18" s="34" t="inlineStr">
+      <c r="Y18" s="34" t="inlineStr">
         <is>
           <t>Część klientów odpada na tym etapie, pojawia się porównywanie ofert.</t>
         </is>
@@ -2655,13 +2542,7 @@
       <c r="X19" s="37" t="n">
         <v>5</v>
       </c>
-      <c r="Y19" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z19" s="37" t="n"/>
-      <c r="AA19" s="34" t="inlineStr">
+      <c r="Y19" s="34" t="inlineStr">
         <is>
           <t>Jeden z najsilniejszych pozytywnych momentów procesu zakupu.</t>
         </is>
@@ -2755,13 +2636,7 @@
       <c r="X20" s="37" t="n">
         <v>5</v>
       </c>
-      <c r="Y20" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z20" s="37" t="n"/>
-      <c r="AA20" s="34" t="inlineStr">
+      <c r="Y20" s="34" t="inlineStr">
         <is>
           <t>Proces zakupu jest oceniany bardzo dobrze.</t>
         </is>
@@ -2870,13 +2745,7 @@
       <c r="X21" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="Y21" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z21" s="37" t="n"/>
-      <c r="AA21" s="34" t="inlineStr">
+      <c r="Y21" s="34" t="inlineStr">
         <is>
           <t>Automatyzacja i raporty BI zapewniają dane o przygotowaniu pojazdu, ale dealerzy nie zawsze czytają informacje ani wykorzystują je w kontakcie z klientem. Brak pewności co do terminów prowadzi do odsyłania klientów do importera i obniża zaufanie do marki.</t>
         </is>
@@ -2980,13 +2849,7 @@
       <c r="X22" s="37" t="n">
         <v>5</v>
       </c>
-      <c r="Y22" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z22" s="37" t="n"/>
-      <c r="AA22" s="34" t="inlineStr">
+      <c r="Y22" s="34" t="inlineStr">
         <is>
           <t>Jeden z najmocniejszych pozytywnych momentów całej podróży klienta.</t>
         </is>
@@ -3090,13 +2953,7 @@
       <c r="X23" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="Y23" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z23" s="37" t="n"/>
-      <c r="AA23" s="34" t="inlineStr">
+      <c r="Y23" s="34" t="inlineStr">
         <is>
           <t>Pakiet może zawierać personalizowany moduł dźwiękowy z imieniem klienta i podziękowaniem za zakup.</t>
         </is>
@@ -3200,13 +3057,7 @@
       <c r="X24" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="Y24" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z24" s="37" t="n"/>
-      <c r="AA24" s="34" t="inlineStr">
+      <c r="Y24" s="34" t="inlineStr">
         <is>
           <t>Planowany mail z podziękowaniem po zakupie auta używanego ma wykorzystywać listę z DSR. Proces ma odtwarzać standard doświadczenia znany ze sprzedaży samochodów nowych.</t>
         </is>
@@ -3295,13 +3146,7 @@
       <c r="X25" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="Y25" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z25" s="37" t="n"/>
-      <c r="AA25" s="34" t="inlineStr">
+      <c r="Y25" s="34" t="inlineStr">
         <is>
           <t>Brak wyraźnych negatywnych lub pozytywnych sygnałów w badaniach.</t>
         </is>
@@ -3390,12 +3235,6 @@
       <c r="X26" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="Y26" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z26" s="37" t="n"/>
     </row>
     <row r="27" ht="36.75" customHeight="1">
       <c r="A27" s="25" t="inlineStr">
@@ -3485,12 +3324,6 @@
       <c r="X27" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="Y27" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z27" s="37" t="n"/>
     </row>
     <row r="28" ht="36.75" customHeight="1">
       <c r="A28" s="25" t="inlineStr">
@@ -3580,12 +3413,6 @@
       <c r="X28" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="Y28" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z28" s="37" t="n"/>
     </row>
     <row r="29" ht="36.75" customHeight="1">
       <c r="A29" s="25" t="inlineStr">
@@ -3670,13 +3497,7 @@
       <c r="X29" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="Y29" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z29" s="37" t="n"/>
-      <c r="AA29" s="34" t="inlineStr">
+      <c r="Y29" s="34" t="inlineStr">
         <is>
           <t>Brak wyraźnych negatywnych lub pozytywnych sygnałów w badaniach.</t>
         </is>
@@ -3780,13 +3601,7 @@
       <c r="X30" s="37" t="n">
         <v>-1</v>
       </c>
-      <c r="Y30" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z30" s="37" t="n"/>
-      <c r="AA30" s="34" t="inlineStr">
+      <c r="Y30" s="34" t="inlineStr">
         <is>
           <t>Program dla klientów lojalnych jest obsługiwany przez doradcę; przy kliencie obecnym w bazie nie są wymagane dodatkowe dokumenty, ewentualnie wykorzystywane są screeny z eMotive.</t>
         </is>
@@ -3875,12 +3690,6 @@
       <c r="X31" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="Y31" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z31" s="37" t="n"/>
     </row>
     <row r="32" ht="36.75" customHeight="1">
       <c r="A32" s="25" t="inlineStr">
@@ -3980,12 +3789,6 @@
       <c r="X32" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="Y32" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z32" s="37" t="n"/>
     </row>
     <row r="33" ht="36.75" customHeight="1">
       <c r="A33" s="27" t="inlineStr">
@@ -4085,13 +3888,7 @@
       <c r="X33" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="Y33" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z33" s="37" t="n"/>
-      <c r="AA33" s="34" t="inlineStr">
+      <c r="Y33" s="34" t="inlineStr">
         <is>
           <t>Funkcjonalny punkt styku, niewiele emocji.</t>
         </is>
@@ -4181,13 +3978,7 @@
       <c r="V34" s="37" t="n"/>
       <c r="W34" s="37" t="n"/>
       <c r="X34" s="37" t="n"/>
-      <c r="Y34" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z34" s="37" t="n"/>
-      <c r="AA34" s="34" t="inlineStr">
+      <c r="Y34" s="34" t="inlineStr">
         <is>
           <t>W zależności od dostępności terminów.</t>
         </is>
@@ -4271,13 +4062,7 @@
       <c r="X35" s="37" t="n">
         <v>-1</v>
       </c>
-      <c r="Y35" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z35" s="37" t="n"/>
-      <c r="AA35" s="34" t="inlineStr">
+      <c r="Y35" s="34" t="inlineStr">
         <is>
           <t>Pojawiają się problemy z dodzwonieniem.</t>
         </is>
@@ -4361,13 +4146,7 @@
       <c r="X36" s="37" t="n">
         <v>-1</v>
       </c>
-      <c r="Y36" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z36" s="37" t="n"/>
-      <c r="AA36" s="34" t="inlineStr">
+      <c r="Y36" s="34" t="inlineStr">
         <is>
           <t>Problem braku odpowiedzi od dealera.</t>
         </is>
@@ -4446,13 +4225,7 @@
       <c r="X37" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="Y37" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z37" s="37" t="n"/>
-      <c r="AA37" s="34" t="inlineStr">
+      <c r="Y37" s="34" t="inlineStr">
         <is>
           <t>Brak silnych sygnałów emocjonalnych.</t>
         </is>
@@ -4546,13 +4319,7 @@
       <c r="X38" s="37" t="n">
         <v>5</v>
       </c>
-      <c r="Y38" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z38" s="37" t="n"/>
-      <c r="AA38" s="34" t="inlineStr">
+      <c r="Y38" s="34" t="inlineStr">
         <is>
           <t>Doradcy serwisowi należą do najlepiej ocenianych elementów doświadczenia.</t>
         </is>
@@ -4646,13 +4413,7 @@
       <c r="X39" s="37" t="n">
         <v>-1</v>
       </c>
-      <c r="Y39" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z39" s="37" t="n"/>
-      <c r="AA39" s="34" t="inlineStr">
+      <c r="Y39" s="34" t="inlineStr">
         <is>
           <t>Klienci oczekują informacji i często jej nie otrzymują.</t>
         </is>
@@ -4746,13 +4507,7 @@
       <c r="X40" s="37" t="n">
         <v>-1</v>
       </c>
-      <c r="Y40" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z40" s="37" t="n"/>
-      <c r="AA40" s="34" t="inlineStr">
+      <c r="Y40" s="34" t="inlineStr">
         <is>
           <t>Kluczowe są czas realizacji i dostępność części.</t>
         </is>
@@ -4846,13 +4601,7 @@
       <c r="X41" s="37" t="n">
         <v>-3</v>
       </c>
-      <c r="Y41" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z41" s="37" t="n"/>
-      <c r="AA41" s="34" t="inlineStr">
+      <c r="Y41" s="34" t="inlineStr">
         <is>
           <t>Najczęściej powtarzający się negatywny temat w CA Service.</t>
         </is>
@@ -4946,12 +4695,6 @@
       <c r="X42" s="37" t="n">
         <v>-1</v>
       </c>
-      <c r="Y42" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z42" s="37" t="n"/>
     </row>
     <row r="43" ht="36.75" customHeight="1">
       <c r="A43" s="27" t="inlineStr">
@@ -5041,13 +4784,7 @@
       <c r="X43" s="37" t="n">
         <v>3</v>
       </c>
-      <c r="Y43" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z43" s="37" t="n"/>
-      <c r="AA43" s="34" t="inlineStr">
+      <c r="Y43" s="34" t="inlineStr">
         <is>
           <t>Jeżeli problem został rozwiązany, emocje ponownie rosną.</t>
         </is>
@@ -5141,12 +4878,6 @@
       <c r="X44" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="Y44" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z44" s="37" t="n"/>
     </row>
     <row r="45" ht="36.75" customHeight="1">
       <c r="A45" s="27" t="inlineStr">
@@ -5236,12 +4967,6 @@
       <c r="X45" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="Y45" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z45" s="37" t="n"/>
     </row>
     <row r="46" ht="36.75" customHeight="1">
       <c r="A46" s="27" t="inlineStr">
@@ -5331,12 +5056,6 @@
       <c r="X46" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="Y46" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z46" s="37" t="n"/>
     </row>
     <row r="47" ht="36.75" customHeight="1">
       <c r="A47" s="27" t="inlineStr">
@@ -5426,13 +5145,7 @@
       <c r="X47" s="37" t="n">
         <v>-1</v>
       </c>
-      <c r="Y47" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z47" s="37" t="n"/>
-      <c r="AA47" s="34" t="inlineStr">
+      <c r="Y47" s="34" t="inlineStr">
         <is>
           <t>Dobrze wykonany buduje relację, brak follow-upu pozostaje niewidoczny dla klienta.</t>
         </is>
@@ -5459,11 +5172,6 @@
           <t>TP030</t>
         </is>
       </c>
-      <c r="Y48" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
     </row>
     <row r="49" ht="36.75" customHeight="1">
       <c r="A49" s="29" t="inlineStr">
@@ -5486,11 +5194,6 @@
           <t>TP031</t>
         </is>
       </c>
-      <c r="Y49" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
     </row>
     <row r="50" ht="36.75" customHeight="1">
       <c r="A50" s="29" t="inlineStr">
@@ -5575,13 +5278,7 @@
       <c r="X50" s="37" t="n">
         <v>-4</v>
       </c>
-      <c r="Y50" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z50" s="37" t="n"/>
-      <c r="AA50" s="34" t="inlineStr">
+      <c r="Y50" s="34" t="inlineStr">
         <is>
           <t>Największe ryzyko utraty zaufania klienta.</t>
         </is>
@@ -5675,12 +5372,6 @@
       <c r="X51" s="37" t="n">
         <v>-2</v>
       </c>
-      <c r="Y51" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z51" s="37" t="n"/>
     </row>
     <row r="52" ht="36.75" customHeight="1">
       <c r="A52" s="29" t="inlineStr">
@@ -5770,12 +5461,6 @@
       <c r="X52" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="Y52" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z52" s="37" t="n"/>
     </row>
     <row r="53" ht="36.75" customHeight="1">
       <c r="A53" s="29" t="inlineStr">
@@ -5865,13 +5550,7 @@
       <c r="X53" s="37" t="n">
         <v>-1</v>
       </c>
-      <c r="Y53" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z53" s="37" t="n"/>
-      <c r="AA53" s="34" t="inlineStr">
+      <c r="Y53" s="34" t="inlineStr">
         <is>
           <t>Kluczowa jest jasna komunikacja i prostota procesu.</t>
         </is>
@@ -5960,13 +5639,7 @@
       <c r="X54" s="37" t="n">
         <v>-1</v>
       </c>
-      <c r="Y54" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z54" s="37" t="n"/>
-      <c r="AA54" s="34" t="inlineStr">
+      <c r="Y54" s="34" t="inlineStr">
         <is>
           <t>Klienci nie czują się wystarczająco doceniani za lojalność.</t>
         </is>
@@ -6075,13 +5748,7 @@
       <c r="X55" s="37" t="n">
         <v>4</v>
       </c>
-      <c r="Y55" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z55" s="37" t="n"/>
-      <c r="AA55" s="34" t="inlineStr">
+      <c r="Y55" s="34" t="inlineStr">
         <is>
           <t>Za skuteczne polecenie klient otrzymuje voucher 700 PLN na przegląd; zakup musi nastąpić w tym samym salonie, a koszt przeglądu ponosi dealer.</t>
         </is>
@@ -6185,12 +5852,6 @@
       <c r="X56" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="Y56" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z56" s="37" t="n"/>
     </row>
     <row r="57" ht="36.75" customHeight="1">
       <c r="A57" s="31" t="inlineStr">
@@ -6290,12 +5951,6 @@
       <c r="X57" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="Y57" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z57" s="37" t="n"/>
     </row>
     <row r="58" ht="36.75" customHeight="1">
       <c r="A58" s="31" t="inlineStr">
@@ -6395,12 +6050,6 @@
       <c r="X58" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="Y58" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z58" s="37" t="n"/>
     </row>
     <row r="59" ht="36.75" customHeight="1">
       <c r="A59" s="31" t="inlineStr">
@@ -6490,13 +6139,7 @@
       <c r="X59" s="37" t="n">
         <v>-0.5</v>
       </c>
-      <c r="Y59" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z59" s="37" t="n"/>
-      <c r="AA59" s="34" t="inlineStr">
+      <c r="Y59" s="34" t="inlineStr">
         <is>
           <t>Powracający klienci oczekują specjalnego traktowania i benefitów.</t>
         </is>
@@ -6600,13 +6243,7 @@
       <c r="X60" s="37" t="n">
         <v>1</v>
       </c>
-      <c r="Y60" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z60" s="37" t="n"/>
-      <c r="AA60" s="34" t="inlineStr">
+      <c r="Y60" s="34" t="inlineStr">
         <is>
           <t>YODA generuje lead na pół roku przed końcem kontraktu, jednak kluczowym problemem pozostaje brak kontaktu ze strony dealera. Zgody TCMR umożliwiają przejęcie kontaktu przez call center, gdy dealer znika, i ustalenie dealera docelowego.</t>
         </is>
@@ -6710,20 +6347,14 @@
       <c r="X61" s="37" t="n">
         <v>0</v>
       </c>
-      <c r="Y61" s="37" t="inlineStr">
-        <is>
-          <t>DEMO</t>
-        </is>
-      </c>
-      <c r="Z61" s="37" t="n"/>
-      <c r="AA61" s="34" t="inlineStr">
+      <c r="Y61" s="34" t="inlineStr">
         <is>
           <t>Zapytanie klienta do banku o finansowanie lub spłatę tworzy lead w YODA do kontaktu przez doradcę. Zgody TCMR pozwalają call center skontaktować się z klientem i ustalić dealera docelowego, gdy dotychczasowy dealer znika.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AB61">
+  <autoFilter ref="A1:Z61">
     <sortState ref="A2:W61">
       <sortCondition ref="A1:A61"/>
     </sortState>

</xml_diff>